<commit_message>
Merge 8518 30 95 into 8518 30 00; add reconciliation check block
TARIC has no subheading 8518 30 95 (confirmed against the client's customs
system), so the headphone lines that the client's HS list split across
8518 30 00 and 8518 30 95 are now a single row 8518 30 00:
120 pcs, 17.35 kg net, 21.87 kg gross, USD 2,870. Summary is now 7 rows,
matching the structure in the declaration.

Added a KONTROLA PROTI DOKLADŮM block to the summary sheet: it compares the
summary totals against the printed packing list, invoice and B/L totals and
shows a difference that must read zero. This makes a mistyped or short row
visible immediately instead of passing silently.

Recalculated: 44 formulas, 0 errors, all four difference cells zero.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThZSGoZoZJt3LPxsuhjXqs
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_PCV_Computers_PCV260729A.xlsx
+++ b/output/HS_Code_Summary_PCV_Computers_PCV260729A.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="220">
   <si>
     <t xml:space="preserve">SOUHRN HS KÓDŮ – PCV Computers, s.r.o.</t>
   </si>
@@ -162,15 +162,6 @@
     <t xml:space="preserve">85183000</t>
   </si>
   <si>
-    <t xml:space="preserve">Sluchátka kombinovaná (náhlavní soupravy s QD-RJ9 konektory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ověřit členění vůči 8518 30 95 – viz list Poznámky.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">85183095</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sluchátka ostatní (bluetooth náhlavní soupravy, kožený náušník, SIP DECT odolná ručka)</t>
   </si>
   <si>
@@ -195,6 +186,27 @@
     <t xml:space="preserve">CELKEM</t>
   </si>
   <si>
+    <t xml:space="preserve">KONTROLA PROTI DOKLADŮM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Netto (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brutto (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hodnota (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Součet tohoto souhrnu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doklady (PL / faktura / B/L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozdíl (musí být 0)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zásilka má jediného odesílatele (Yealink Xiamen), proto je celý souhrn jedním blokem; HS kódy jsou sloučeny na unikátní řádky.</t>
   </si>
   <si>
@@ -210,6 +222,9 @@
     <t xml:space="preserve">Žádná obchodní sleva není v dokladech uvedena – poměrné rozpuštění slevy se neuplatňuje.</t>
   </si>
   <si>
+    <t xml:space="preserve">Kontrolní blok výše musí vykazovat nulový rozdíl proti packing listu, faktuře a B/L – jinak je v deklaraci chyba.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part Number</t>
   </si>
   <si>
@@ -225,9 +240,6 @@
     <t xml:space="preserve">HS kód (klient)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hodnota (USD)</t>
-  </si>
-  <si>
     <t xml:space="preserve">HS kód dle faktury Yealink</t>
   </si>
   <si>
@@ -630,16 +642,16 @@
     <t xml:space="preserve">   • PSU-5V/2A: klient 8504 40 60 × Yealink 8504 40 95 90.</t>
   </si>
   <si>
-    <t xml:space="preserve">4) ČLENĚNÍ 8518 30 – KE KONTROLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Klient uvádí dva kódy v rámci téže položky: 8518 30 00 (YHS34 / YHS36) a 8518 30 95 (BH70, BH71, náušník, W57R).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Obě podpoložky jsou v souhrnu ponechány odděleně tak, jak je klient dodal.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">→ Před podáním celního prohlášení ověřte platné členění 8518 30 v TARIC; sazebně jsou obě v rámci ITA bezcelní.</t>
+    <t xml:space="preserve">4) ČLENĚNÍ 8518 30 – VYŘEŠENO, SLOUČENO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klientův seznam uváděl dva kódy: 8518 30 00 (YHS34 / YHS36) a 8518 30 95 (BH70, BH71, náušník, W57R).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Podpoložka 8518 30 95 v TARIC neexistuje – potvrzeno klientem podle celního systému.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Obě skupiny jsou proto sloučeny do jediného řádku 8518 30 00 (DK 90): 80 ks, 17,35 kg netto, 21,87 kg brutto, 2 870 USD.</t>
   </si>
   <si>
     <t xml:space="preserve">5) ANTIDUMPING</t>
@@ -734,16 +746,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="9"/>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
+      <i val="true"/>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -824,7 +836,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -893,15 +905,51 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1161,7 +1209,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -1497,19 +1545,19 @@
       </c>
       <c r="D20" s="7" t="n">
         <f aca="false">SUMIFS(Položky!$G$2:$G$38,Položky!$E$2:$E$38,$B20)</f>
-        <v>7.58</v>
+        <v>17.35</v>
       </c>
       <c r="E20" s="7" t="n">
         <f aca="false">SUMIFS(Položky!$H$2:$H$38,Položky!$E$2:$E$38,$B20)</f>
-        <v>10.2</v>
+        <v>21.87</v>
       </c>
       <c r="F20" s="8" t="n">
         <f aca="false">SUMIFS(Položky!$F$2:$F$38,Položky!$E$2:$E$38,$B20)</f>
-        <v>40</v>
+        <v>120</v>
       </c>
       <c r="G20" s="7" t="n">
         <f aca="false">SUMIFS(Položky!$I$2:$I$38,Položky!$E$2:$E$38,$B20)</f>
-        <v>780</v>
+        <v>2870</v>
       </c>
       <c r="H20" s="5" t="s">
         <v>12</v>
@@ -1525,192 +1573,245 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="11" t="n">
         <f aca="false">SUMIFS(Položky!$G$2:$G$38,Položky!$E$2:$E$38,$B21)</f>
-        <v>9.77</v>
-      </c>
-      <c r="E21" s="7" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="E21" s="11" t="n">
         <f aca="false">SUMIFS(Položky!$H$2:$H$38,Položky!$E$2:$E$38,$B21)</f>
-        <v>11.67</v>
-      </c>
-      <c r="F21" s="8" t="n">
+        <v>42.71</v>
+      </c>
+      <c r="F21" s="12" t="n">
         <f aca="false">SUMIFS(Položky!$F$2:$F$38,Položky!$E$2:$E$38,$B21)</f>
-        <v>80</v>
-      </c>
-      <c r="G21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="11" t="n">
         <f aca="false">SUMIFS(Položky!$I$2:$I$38,Položky!$E$2:$E$38,$B21)</f>
-        <v>2090</v>
-      </c>
-      <c r="H21" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="H21" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="I21" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K21" s="5" t="s">
+      <c r="I21" s="10" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="B22" s="10" t="s">
+      <c r="J21" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="K21" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="11" t="n">
-        <f aca="false">SUMIFS(Položky!$G$2:$G$38,Položky!$E$2:$E$38,$B22)</f>
-        <v>31.6</v>
-      </c>
-      <c r="E22" s="11" t="n">
-        <f aca="false">SUMIFS(Položky!$H$2:$H$38,Položky!$E$2:$E$38,$B22)</f>
-        <v>42.71</v>
-      </c>
-      <c r="F22" s="12" t="n">
-        <f aca="false">SUMIFS(Položky!$F$2:$F$38,Položky!$E$2:$E$38,$B22)</f>
-        <v>2</v>
-      </c>
-      <c r="G22" s="11" t="n">
-        <f aca="false">SUMIFS(Položky!$I$2:$I$38,Položky!$E$2:$E$38,$B22)</f>
-        <v>640</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="I22" s="10" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="J22" s="10" t="s">
+      <c r="D22" s="15" t="n">
+        <f aca="false">SUM(D15:D21)</f>
+        <v>1142.99</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <f aca="false">SUM(E15:E21)</f>
+        <v>1391.49</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <f aca="false">SUM(F15:F21)</f>
+        <v>1416</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <f aca="false">SUM(G15:G21)</f>
+        <v>69882</v>
+      </c>
+      <c r="H22" s="13"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C24" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="K22" s="9" t="s">
+      <c r="D24" s="18" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="13" t="s">
+      <c r="E24" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="15" t="n">
-        <f aca="false">SUM(D15:D22)</f>
+      <c r="F24" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C25" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D25" s="21" t="n">
+        <f aca="false">D22</f>
         <v>1142.99</v>
       </c>
-      <c r="E23" s="15" t="n">
-        <f aca="false">SUM(E15:E22)</f>
+      <c r="E25" s="21" t="n">
+        <f aca="false">E22</f>
         <v>1391.49</v>
       </c>
-      <c r="F23" s="16" t="n">
-        <f aca="false">SUM(F15:F22)</f>
+      <c r="F25" s="22" t="n">
+        <f aca="false">F22</f>
         <v>1416</v>
       </c>
-      <c r="G23" s="15" t="n">
-        <f aca="false">SUM(G15:G22)</f>
+      <c r="G25" s="21" t="n">
+        <f aca="false">G22</f>
         <v>69882</v>
       </c>
-      <c r="H23" s="13"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="13"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
+      <c r="C26" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" s="21" t="n">
+        <v>1142.99</v>
+      </c>
+      <c r="E26" s="21" t="n">
+        <v>1391.49</v>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>1416</v>
+      </c>
+      <c r="G26" s="21" t="n">
+        <v>69882</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
+      <c r="C27" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
+      <c r="D27" s="24" t="n">
+        <f aca="false">D25-D26</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="24" t="n">
+        <f aca="false">E25-E26</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="25" t="n">
+        <f aca="false">F25-F26</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <f aca="false">G25-G26</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="26"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="26"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="26"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="26"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="26"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="26"/>
+      <c r="J33" s="26"/>
+      <c r="K33" s="26"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="26"/>
+      <c r="J34" s="26"/>
+      <c r="K34" s="26"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A27:K27"/>
-    <mergeCell ref="A28:K28"/>
+  <mergeCells count="6">
     <mergeCell ref="A29:K29"/>
+    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A31:K31"/>
+    <mergeCell ref="A32:K32"/>
+    <mergeCell ref="A33:K33"/>
+    <mergeCell ref="A34:K34"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1743,19 +1844,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>26</v>
@@ -1767,21 +1868,21 @@
         <v>25</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>39</v>
@@ -1802,18 +1903,18 @@
         <v>980</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>36</v>
@@ -1834,88 +1935,88 @@
         <v>1176</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="F4" s="12" t="n">
+      <c r="A4" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="7" t="n">
         <v>3.61</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H4" s="7" t="n">
         <v>4.32</v>
       </c>
-      <c r="I4" s="11" t="n">
+      <c r="I4" s="7" t="n">
         <v>640</v>
       </c>
-      <c r="J4" s="10" t="s">
-        <v>80</v>
+      <c r="J4" s="6" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" s="12" t="n">
+      <c r="A5" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="7" t="n">
         <v>1.34</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="7" t="n">
         <v>1.53</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I5" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="J5" s="10" t="s">
-        <v>80</v>
+      <c r="J5" s="6" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>50</v>
@@ -1930,24 +2031,24 @@
         <v>150</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F7" s="12" t="n">
         <v>2</v>
@@ -1962,18 +2063,18 @@
         <v>640</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>43</v>
@@ -1994,18 +2095,18 @@
         <v>200</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>39</v>
@@ -2026,18 +2127,18 @@
         <v>3000</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>33</v>
@@ -2058,18 +2159,18 @@
         <v>300</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>36</v>
@@ -2090,18 +2191,18 @@
         <v>2300</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>36</v>
@@ -2122,18 +2223,18 @@
         <v>6200</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>36</v>
@@ -2154,18 +2255,18 @@
         <v>5400</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>36</v>
@@ -2186,18 +2287,18 @@
         <v>6000</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>36</v>
@@ -2218,18 +2319,18 @@
         <v>3150</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>36</v>
@@ -2250,18 +2351,18 @@
         <v>2250</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>115</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>36</v>
@@ -2282,18 +2383,18 @@
         <v>4550</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>36</v>
@@ -2314,18 +2415,18 @@
         <v>510</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>36</v>
@@ -2346,18 +2447,18 @@
         <v>1360</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>36</v>
@@ -2378,18 +2479,18 @@
         <v>265</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>36</v>
@@ -2410,18 +2511,18 @@
         <v>1950</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>127</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>36</v>
@@ -2442,18 +2543,18 @@
         <v>2200</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>43</v>
@@ -2474,18 +2575,18 @@
         <v>228</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>36</v>
@@ -2506,18 +2607,18 @@
         <v>120</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>41</v>
@@ -2538,18 +2639,18 @@
         <v>600</v>
       </c>
       <c r="J25" s="10" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>41</v>
@@ -2570,24 +2671,24 @@
         <v>600</v>
       </c>
       <c r="J26" s="10" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F27" s="12" t="n">
         <v>10</v>
@@ -2602,18 +2703,18 @@
         <v>700</v>
       </c>
       <c r="J27" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>36</v>
@@ -2634,18 +2735,18 @@
         <v>740</v>
       </c>
       <c r="J28" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>36</v>
@@ -2666,18 +2767,18 @@
         <v>1800</v>
       </c>
       <c r="J29" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B30" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="C30" s="10" t="s">
         <v>156</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>152</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>36</v>
@@ -2698,18 +2799,18 @@
         <v>4300</v>
       </c>
       <c r="J30" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>36</v>
@@ -2730,18 +2831,18 @@
         <v>14400</v>
       </c>
       <c r="J31" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>36</v>
@@ -2762,18 +2863,18 @@
         <v>650</v>
       </c>
       <c r="J32" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>36</v>
@@ -2794,18 +2895,18 @@
         <v>970</v>
       </c>
       <c r="J33" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>36</v>
@@ -2826,18 +2927,18 @@
         <v>173</v>
       </c>
       <c r="J34" s="10" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>46</v>
@@ -2858,18 +2959,18 @@
         <v>220</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>46</v>
@@ -2890,18 +2991,18 @@
         <v>160</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>46</v>
@@ -2922,18 +3023,18 @@
         <v>220</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>46</v>
@@ -2954,14 +3055,14 @@
         <v>180</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14"/>
       <c r="B39" s="14"/>
       <c r="C39" s="14" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D39" s="13"/>
       <c r="E39" s="14"/>
@@ -2984,13 +3085,13 @@
       <c r="J39" s="14"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18" t="s">
-        <v>178</v>
+      <c r="A41" s="27" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="18" t="s">
-        <v>179</v>
+      <c r="A42" s="27" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -3018,428 +3119,428 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
+      <c r="A3" s="28" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
-        <v>182</v>
-      </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
+      <c r="A4" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
-        <v>183</v>
-      </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
+      <c r="A5" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
+      <c r="A6" s="29" t="s">
+        <v>188</v>
+      </c>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>185</v>
-      </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
+      <c r="A7" s="29" t="s">
+        <v>189</v>
+      </c>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
-        <v>186</v>
-      </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
+      <c r="A9" s="28" t="s">
+        <v>190</v>
+      </c>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
-        <v>187</v>
-      </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
+      <c r="A10" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
+      <c r="A11" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
+      <c r="A12" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>190</v>
-      </c>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
+      <c r="A13" s="29" t="s">
+        <v>194</v>
+      </c>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>191</v>
-      </c>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
+      <c r="A14" s="29" t="s">
+        <v>195</v>
+      </c>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
-        <v>192</v>
-      </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
+      <c r="A15" s="29" t="s">
+        <v>196</v>
+      </c>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
+      <c r="A17" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
-        <v>194</v>
-      </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
+      <c r="A18" s="29" t="s">
+        <v>198</v>
+      </c>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="29"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
+      <c r="A19" s="29" t="s">
+        <v>199</v>
+      </c>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
-        <v>196</v>
-      </c>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
+      <c r="A20" s="29" t="s">
+        <v>200</v>
+      </c>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
-        <v>197</v>
-      </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
+      <c r="A21" s="29" t="s">
+        <v>201</v>
+      </c>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
-        <v>198</v>
-      </c>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
+      <c r="A22" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
-        <v>199</v>
-      </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
+      <c r="A23" s="29" t="s">
+        <v>203</v>
+      </c>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
-        <v>200</v>
-      </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
+      <c r="A24" s="29" t="s">
+        <v>204</v>
+      </c>
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="29"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
-        <v>201</v>
-      </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20"/>
+      <c r="A25" s="29" t="s">
+        <v>205</v>
+      </c>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="29"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
-        <v>202</v>
-      </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
+      <c r="A27" s="28" t="s">
+        <v>206</v>
+      </c>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
-        <v>203</v>
-      </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
+      <c r="A28" s="29" t="s">
+        <v>207</v>
+      </c>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="20"/>
+      <c r="A29" s="29" t="s">
+        <v>208</v>
+      </c>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
-        <v>205</v>
-      </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
-      <c r="H30" s="20"/>
+      <c r="A30" s="29" t="s">
+        <v>209</v>
+      </c>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="29"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
+      <c r="A32" s="28" t="s">
+        <v>210</v>
+      </c>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
-        <v>207</v>
-      </c>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
+      <c r="A33" s="29" t="s">
+        <v>211</v>
+      </c>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
+      <c r="A34" s="29" t="s">
+        <v>212</v>
+      </c>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
-        <v>209</v>
-      </c>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
+      <c r="A35" s="29" t="s">
+        <v>213</v>
+      </c>
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="29"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="B37" s="19"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
+      <c r="A37" s="28" t="s">
+        <v>214</v>
+      </c>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="28"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
-        <v>211</v>
-      </c>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="20"/>
-      <c r="G38" s="20"/>
-      <c r="H38" s="20"/>
+      <c r="A38" s="29" t="s">
+        <v>215</v>
+      </c>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="20" t="s">
-        <v>212</v>
-      </c>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
+      <c r="A39" s="29" t="s">
+        <v>216</v>
+      </c>
+      <c r="B39" s="29"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="29"/>
+      <c r="F39" s="29"/>
+      <c r="G39" s="29"/>
+      <c r="H39" s="29"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="20" t="s">
-        <v>213</v>
-      </c>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
+      <c r="A40" s="29" t="s">
+        <v>217</v>
+      </c>
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="20"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="20"/>
-      <c r="H41" s="20"/>
+      <c r="A41" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="29"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="20" t="s">
-        <v>215</v>
-      </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
+      <c r="A42" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="35">

</xml_diff>